<commit_message>
fix: polish category page styling to match original Tory Burch design
Center H1/H2 headings, add section dividers between categories,
fix full-width grid layout on desktop, refine cards-product CSS
with design tokens and correct aspect ratios. Restructure shoes,
clothing, and accessories pages into proper cards-product blocks.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-category-page.report.xlsx
+++ b/tools/importer/reports/import-category-page.report.xlsx
@@ -73,7 +73,7 @@
     <t>category-page</t>
   </si>
   <si>
-    <t>2026-04-13T17:00:40.242Z</t>
+    <t>2026-04-13T17:20:17.621Z</t>
   </si>
   <si>
     <t>Designer Bags | Handbags &amp; Purses for Women | Tory Burch</t>
@@ -91,7 +91,7 @@
     <t>en-us/accessories/view-all</t>
   </si>
   <si>
-    <t>2026-04-13T17:01:11.672Z</t>
+    <t>2026-04-13T17:20:46.494Z</t>
   </si>
   <si>
     <t>Designer Accessories | Fashion Accessories for Women | Tory Burch</t>
@@ -106,7 +106,7 @@
     <t>en-us/clothing/view-all</t>
   </si>
   <si>
-    <t>2026-04-13T17:01:01.278Z</t>
+    <t>2026-04-13T17:20:36.964Z</t>
   </si>
   <si>
     <t>Shop All Women's Designer Fashion Collection | Tory Burch</t>
@@ -121,7 +121,7 @@
     <t>en-us/shoes/view-all</t>
   </si>
   <si>
-    <t>2026-04-13T17:00:50.473Z</t>
+    <t>2026-04-13T17:20:26.710Z</t>
   </si>
   <si>
     <t>Women's Designer Shoes | Tory Burch</t>

</xml_diff>